<commit_message>
Sprint 3 - Ultimos ajustes
</commit_message>
<xml_diff>
--- a/matriz_rastreabilidade.xlsx
+++ b/matriz_rastreabilidade.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valores Limite" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura Total" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela Inversa" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3 - CSV e Nulos" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -131,7 +132,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -145,11 +146,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -203,6 +232,8 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -587,13 +618,13 @@
           <t>SPRINT 1 — Autenticação (/auth)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1255,10 +1286,10 @@
           <t>Cobertura de Testes — Sprint 3 Final</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1500,6 +1531,18 @@
       <c r="E10" s="18" t="inlineStr">
         <is>
           <t>98.17%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Total de Testes</t>
+        </is>
+      </c>
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>138 / 138 passaram</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1543,8 +1586,8 @@
           <t>Tabela Inversa — Requisito → Casos de Teste</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1678,7 +1721,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>TU25, TU26, TU27, TU28</t>
+          <t>TU25, TU26, TU27, TU28, TU129, TU130, TU131, TU132, TU133, TU134, TU135, TU136, TU137, TU138</t>
         </is>
       </c>
     </row>
@@ -1951,12 +1994,784 @@
       <c r="C25" s="6" t="inlineStr">
         <is>
           <t>TU118, TU119, TU120, TU121, TU122</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>RN-24</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>Validação de campos nulos/vazios em ervas</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>TU123, TU124, TU125, TU126, TU127, TU128</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SPRINT 3 — Valores Nulos, Vazios e Controlo de Acesso CSV</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TU123</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome null rejeitado</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>{ name: null, ... }</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome inválido"</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>TU124</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome undefined rejeitado</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>{ name: undefined, ... }</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome inválido"</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>TU125</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome com espaços rejeitado</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>{ name: "   ", ... }</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome inválido"</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>TU126</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome científico null</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: null, ... }</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome científico inválido"</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TU127</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome científico undefined</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: undefined, ... }</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome científico inválido"</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>TU128</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome científico com espaços</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: "   ", ... }</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome científico inválido"</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TU129</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>RN-07: Administrador pode importar</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Administrador" }</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>{ success: 1, failed: 0 }</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>TU130</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: Tecnico não pode importar</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Tecnico" }</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Apenas o Administrador pode importar"</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>TU131</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: Responsavel não pode importar</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Responsavel" }</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Apenas o Administrador pode importar"</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>TU132</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: sem perfil não pode importar</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: null }</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Apenas o Administrador pode importar"</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>TU133</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com nome null</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>{ name: null, ... }</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1, errors[0]: 'Nome inválido' }</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>TU134</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com nome vazio</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>{ name: "", ... }</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1, errors[0]: 'Nome inválido' }</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>TU135</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com scientificName null</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: null, ... }</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1, errors[0]: 'Nome científico inválido' }</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>TU136</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com cycledays null</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>{ cycledays: null, ... }</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>TU137</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>RN-07: CSV misto (nulos + válidos)</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>PE (classe mista)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>1 linha null + 1 linha válida</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>{ success: 1, failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>TU138</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: CSV com todas as linhas nulas</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>1 linha com todos os campos null</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>{ success: 0, failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1987,13 +2802,13 @@
           <t>SPRINT 2 — Ervas Aromáticas (/herbs)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -2658,13 +3473,13 @@
           <t>SPRINT 2 — Planos de Cultivo (/plans)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -3959,13 +4774,13 @@
           <t>SPRINT 3 — Alertas (/alerts)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -4924,13 +5739,13 @@
           <t>SPRINT 3 — Medições (/measurements)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -5637,13 +6452,13 @@
           <t>SPRINT 3 — Lotes (/batches)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -6434,13 +7249,13 @@
           <t>SPRINT 3 — Automação (/automation)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -7756,12 +8571,12 @@
           <t>Tabela de Valores Limite — Todos os Sprints</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="22" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Sprint 4 - Matriz .md e .xlsx atualizados
</commit_message>
<xml_diff>
--- a/matriz_rastreabilidade.xlsx
+++ b/matriz_rastreabilidade.xlsx
@@ -19,6 +19,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cobertura Total" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabela Inversa" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3 - CSV e Nulos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4 - Auth" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4 - Herbs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4 - Plans" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -234,6 +237,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1270,7 +1277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1283,7 +1290,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cobertura de Testes — Sprint 3 Final</t>
+          <t>Cobertura de Testes — Sprint 4 Final</t>
         </is>
       </c>
       <c r="B1" s="21" t="n"/>
@@ -1555,6 +1562,160 @@
       <c r="B13" s="20" t="inlineStr">
         <is>
           <t>122 / 122 passaram</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>--- Sprint 4 (Integração) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>authController.js</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>authRoutes.js</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>herbsRoutes.js</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>plansRoutes.js</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>85.79%</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>91.48%</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>79.06%</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>86.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Total de Testes</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>172 / 172 passaram</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2011,6 +2172,108 @@
       <c r="C26" s="16" t="inlineStr">
         <is>
           <t>TU123, TU124, TU125, TU126, TU127, TU128</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="25" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>RN-01 (integração)</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Registo de utilizadores</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>TI01a, TI01b, TI01c, TI01d, TI01e, TI01f, TI01g, TI01h</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>RN-03 (integração)</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Login de utilizadores</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>TI02a, TI02b, TI02c, TI02d, TI02e</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="25" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>RN-04 (integração)</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Refresh token</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>TI03a, TI03b, TI03c</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="25" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>RN-05 (integração)</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Criação de ervas</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>TI04a, TI04b, TI04c, TI04d, TI04e</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="25" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>RN-07 (integração)</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Importação CSV</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>TI05a, TI05b, TI05c, TI05d</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="25" customHeight="1">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>RN-08 (integração)</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>Planos de cultivo</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>TI06a, TI06b, TI06c, TI06d, TI06e, TI06f, TI06g, TI06h, TI06i</t>
         </is>
       </c>
     </row>
@@ -2047,6 +2310,761 @@
           <t>SPRINT 3 — Valores Nulos, Vazios e Controlo de Acesso CSV</t>
         </is>
       </c>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>TU123</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome null rejeitado</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>{ name: null, ... }</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome inválido"</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>TU124</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome undefined rejeitado</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>{ name: undefined, ... }</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome inválido"</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>TU125</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome com espaços rejeitado</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>{ name: "   ", ... }</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome inválido"</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>TU126</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome científico null</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: null, ... }</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome científico inválido"</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TU127</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome científico undefined</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: undefined, ... }</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome científico inválido"</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>TU128</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>RN-24: nome científico com espaços</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: "   ", ... }</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Nome científico inválido"</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TU129</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>RN-07: Administrador pode importar</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Administrador" }</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>{ success: 1, failed: 0 }</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>TU130</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: Tecnico não pode importar</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Tecnico" }</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Apenas o Administrador pode importar"</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>TU131</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: Responsavel não pode importar</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Responsavel" }</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Apenas o Administrador pode importar"</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>TU132</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: sem perfil não pode importar</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: null }</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Erro: "Apenas o Administrador pode importar"</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>TU133</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com nome null</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>{ name: null, ... }</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1, errors[0]: 'Nome inválido' }</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>TU134</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com nome vazio</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>{ name: "", ... }</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1, errors[0]: 'Nome inválido' }</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>TU135</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com scientificName null</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>{ scientificName: null, ... }</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1, errors[0]: 'Nome científico inválido' }</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>TU136</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: linha CSV com cycledays null</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>{ cycledays: null, ... }</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>{ failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>TU137</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>RN-07: CSV misto (nulos + válidos)</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>PE (classe mista)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>1 linha null + 1 linha válida</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>{ success: 1, failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>TU138</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: CSV com todas as linhas nulas</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>1 linha com todos os campos null</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>{ success: 0, failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Perfil Administrador</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SPRINT 4 — Testes de Integração: Autenticação (/auth)</t>
+        </is>
+      </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
@@ -2098,56 +3116,811 @@
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>TU123</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>RN-24: nome null rejeitado</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TI01a</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>RN-01: registo válido Tecnico</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>{ username: "tecnico1", password: "123456", role: "Tecnico" }</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>201 - { username: "tecnico1", role: "Tecnico" }</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TI01b</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>RN-01: registo válido Responsavel</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>{ username: "responsavel1", password: "123456", role: "Responsavel" }</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TI01c</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>RN-01: registo válido Administrador</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>{ username: "admin1", password: "123456", role: "Administrador" }</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>TI01d</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>RN-01: perfil inválido</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>{ username: "hacker", password: "123456", role: "Hacker" }</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>400 - { error: "..." }</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TI01e</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>RN-02: username duplicado</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>{ username: "duplicado", password: "123456", role: "Tecnico" }</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Utilizador já registado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>TI01f</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>RN-02: body vazio</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>TI01g</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>RN-02: sem Content-Type</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>form-urlencoded</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>TI01h</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>RN-02: método GET não permitido</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>GET /auth/register</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TI02a</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>RN-03: login válido devolve tokens</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/login</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>{ username: "loginuser", password: "123456" }</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>200 - { token: "...", refreshToken: "..." }</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Utilizador registado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>TI02b</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>RN-03: password errada</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/login</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>{ username: "loginuser", password: "errada" }</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Utilizador registado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>TI02c</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>RN-03: username inexistente</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/login</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>{ username: "naoexiste", password: "123456" }</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>TI02d</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>RN-03: body vazio</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/login</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>TI02e</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>RN-03: username vazio</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/login</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>{ username: "", password: "123456" }</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>TI03a</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>RN-04: refresh token válido</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>POST /auth/refresh</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>{ refreshToken: "&lt;token válido&gt;" }</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>200 - { token: "..." }</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Utilizador logado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>TI03b</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>RN-04: refresh token inválido</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/refresh</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>{ refreshToken: "token_invalido" }</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>TI03c</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>RN-04: sem refresh token</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/refresh</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SPRINT 4 — Testes de Integração: Ervas (/herbs)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TI04a</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>RN-05: criação válida</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>POST /herbs</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>{ name: null, ... }</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Erro: "Nome inválido"</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Nenhuma</t>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>{ name: "Hortelã", scientificName: "Mentha spicata", cycledays: 90, ... }</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>201 - { id: ..., name: "Hortelã" }</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>TU124</t>
+          <t>TI04b</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>RN-24: nome undefined rejeitado</t>
+          <t>RN-05: nome vazio</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -2157,7 +3930,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Unidade</t>
+          <t>Integração</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -2167,71 +3940,71 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>{ name: undefined, ... }</t>
+          <t>{ name: "", ... }</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Erro: "Nome inválido"</t>
+          <t>400 - { error: "..." }</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Nenhuma</t>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>TU125</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>RN-24: nome com espaços rejeitado</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>TI04c</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>RN-06: cycledays = 0</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>POST /herbs</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>{ name: "   ", ... }</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Erro: "Nome inválido"</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Nenhuma</t>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>VL (abaixo limite inferior)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>{ cycledays: 0, ... }</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>TU126</t>
+          <t>TI04d</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>RN-24: nome científico null</t>
+          <t>RN-05: body vazio</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2241,7 +4014,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Unidade</t>
+          <t>Integração</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -2251,39 +4024,500 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>{ scientificName: null, ... }</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Erro: "Nome científico inválido"</t>
+          <t>400</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Nenhuma</t>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TI04e</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>RN-05: GET devolve lista</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>GET /herbs</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>200 - Array</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TI05a</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>RN-07: importação válida por Administrador</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Administrador" }</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>200 - { success: 1, failed: 0 }</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>TI05b</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: importação por Tecnico</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [...], userRole: "Tecnico" }</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>TI05c</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>RN-07: ficheiro vazio</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>{ rows: [], userRole: "Administrador" }</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TI05d</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>RN-07: linhas mistas</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>POST /herbs/import</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe mista)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>1 válida + 1 inválida</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>200 - { success: 1, failed: 1 }</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SPRINT 4 — Testes de Integração: Planos (/plans)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TI06a</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>RN-08: plano regular válido</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>POST /plans</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>{ type: "regular", ... }</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>201 - { type: "regular" }</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TI06b</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>RN-08: plano emergencia válido</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>POST /plans</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>{ type: "emergencia", ... }</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TI06c</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>RN-08: pontual com autorização</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>POST /plans</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>{ type: "pontual", authorizedBy: "responsavel1", ... }</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>201 - { authorizedBy: "responsavel1" }</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>TI06d</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>RN-08: pontual sem autorização</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>POST /plans</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>PE (classe inválida)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>{ type: "pontual", authorizedBy: null, ... }</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>400 - { error: "..." }</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>TU127</t>
+          <t>TI06e</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>RN-24: nome científico undefined</t>
+          <t>RN-08: tipo inválido</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>POST /herbs</t>
+          <t>POST /plans</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Unidade</t>
+          <t>Integração</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2293,123 +4527,123 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>{ scientificName: undefined, ... }</t>
+          <t>{ type: "invalido", ... }</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Erro: "Nome científico inválido"</t>
+          <t>400</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Nenhuma</t>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>TU128</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>RN-24: nome científico com espaços</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>{ scientificName: "   ", ... }</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Erro: "Nome científico inválido"</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Nenhuma</t>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>TI06f</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>RN-09: temperatura fora dos limites</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>POST /plans</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>VL (abaixo limite inferior)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>{ minTemp: 17, ... }</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>TU129</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>RN-07: Administrador pode importar</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>PE (classe válida)</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>{ rows: [...], userRole: "Administrador" }</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>{ success: 1, failed: 0 }</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Nenhuma</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>TI06g</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>RN-10: humidade fora dos limites</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>POST /plans</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>VL (abaixo limite inferior)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>{ minHumidity: 39, ... }</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>TU130</t>
+          <t>TI06h</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>RN-07: Tecnico não pode importar</t>
+          <t>RN-08: body vazio</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>POST /herbs/import</t>
+          <t>POST /plans</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Unidade</t>
+          <t>Integração</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -2419,353 +4653,59 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>{ rows: [...], userRole: "Tecnico" }</t>
+          <t>{}</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Erro: "Apenas o Administrador pode importar"</t>
+          <t>400</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Nenhuma</t>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>TU131</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: Responsavel não pode importar</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>{ rows: [...], userRole: "Responsavel" }</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Erro: "Apenas o Administrador pode importar"</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Nenhuma</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>TU132</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: sem perfil não pode importar</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>{ rows: [...], userRole: null }</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Erro: "Apenas o Administrador pode importar"</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Nenhuma</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>TU133</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: linha CSV com nome null</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>{ name: null, ... }</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>{ failed: 1, errors[0]: 'Nome inválido' }</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Perfil Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>TU134</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: linha CSV com nome vazio</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>{ name: "", ... }</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>{ failed: 1, errors[0]: 'Nome inválido' }</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Perfil Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>TU135</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: linha CSV com scientificName null</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>{ scientificName: null, ... }</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>{ failed: 1, errors[0]: 'Nome científico inválido' }</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Perfil Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>TU136</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: linha CSV com cycledays null</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>{ cycledays: null, ... }</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>{ failed: 1 }</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Perfil Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>TU137</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>RN-07: CSV misto (nulos + válidos)</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>PE (classe mista)</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>1 linha null + 1 linha válida</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>{ success: 1, failed: 1 }</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>Perfil Administrador</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>TU138</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>RN-07: CSV com todas as linhas nulas</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>POST /herbs/import</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Unidade</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>PE (classe inválida)</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>1 linha com todos os campos null</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>{ success: 0, failed: 1 }</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Perfil Administrador</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TI06i</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>RN-08: GET devolve lista</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>GET /plans</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Integração</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>PE (classe válida)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>200 - Array</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Servidor a correr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sprint 6 - Ficheiro .xlsx atualizado
</commit_message>
<xml_diff>
--- a/matriz_rastreabilidade.xlsx
+++ b/matriz_rastreabilidade.xlsx
@@ -24,6 +24,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 4 - Plans" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5 - White Box" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 5 - White Box1" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6 - Stubs e Mocks" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 6 - Stubs e Mocks1" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -85,7 +87,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -172,6 +174,36 @@
         <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1F5EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAECE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F6E56"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001D9E75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00993C1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D85A30"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -219,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -310,6 +342,36 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1348,7 +1410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1933,6 +1995,260 @@
       <c r="B34" s="20" t="inlineStr">
         <is>
           <t>208 / 208 passaram</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>--- Sprint 6 (Stubs e Mocks) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>monitoringService.js</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>temperatureGateway.js</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>notificationGateway.js</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL FINAL</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>71.34%</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>91.7%</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>52.23%</t>
+        </is>
+      </c>
+      <c r="E40" s="24" t="inlineStr">
+        <is>
+          <t>72.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>Total de Testes</t>
+        </is>
+      </c>
+      <c r="B42" s="20" t="inlineStr">
+        <is>
+          <t>219 / 219 passaram</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>--- Sprint 6 (Stubs e Mocks) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>monitoringService.js</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>temperatureGateway.js</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>notificationGateway.js</t>
+        </is>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL FINAL</t>
+        </is>
+      </c>
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>71.34%</t>
+        </is>
+      </c>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>91.7%</t>
+        </is>
+      </c>
+      <c r="D48" s="24" t="inlineStr">
+        <is>
+          <t>52.23%</t>
+        </is>
+      </c>
+      <c r="E48" s="24" t="inlineStr">
+        <is>
+          <t>72.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>Total de Testes</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>219 / 219 passaram</t>
         </is>
       </c>
     </row>
@@ -1950,7 +2266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2661,6 +2977,74 @@
       <c r="C42" s="25" t="inlineStr">
         <is>
           <t>WB26, WB27, WB28, WB29, WB35</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="25" customHeight="1">
+      <c r="A43" s="36" t="inlineStr">
+        <is>
+          <t>RN-25</t>
+        </is>
+      </c>
+      <c r="B43" s="36" t="inlineStr">
+        <is>
+          <t>Monitorização automática de temperatura (Stub)</t>
+        </is>
+      </c>
+      <c r="C43" s="36" t="inlineStr">
+        <is>
+          <t>SP01a, SP01b, SP01c, SP01d, SP01e</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="25" customHeight="1">
+      <c r="A44" s="37" t="inlineStr">
+        <is>
+          <t>RN-26</t>
+        </is>
+      </c>
+      <c r="B44" s="37" t="inlineStr">
+        <is>
+          <t>Envio de notificações de alertas (Mock)</t>
+        </is>
+      </c>
+      <c r="C44" s="37" t="inlineStr">
+        <is>
+          <t>SP02a, SP02b, SP02c, SP02d, SP02e, SP02f</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="25" customHeight="1">
+      <c r="A45" s="36" t="inlineStr">
+        <is>
+          <t>RN-25</t>
+        </is>
+      </c>
+      <c r="B45" s="36" t="inlineStr">
+        <is>
+          <t>Monitorização automática de temperatura</t>
+        </is>
+      </c>
+      <c r="C45" s="36" t="inlineStr">
+        <is>
+          <t>SP01a, SP01b, SP01c, SP01d, SP01e</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="25" customHeight="1">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>RN-26</t>
+        </is>
+      </c>
+      <c r="B46" s="37" t="inlineStr">
+        <is>
+          <t>Envio de notificações de alertas</t>
+        </is>
+      </c>
+      <c r="C46" s="37" t="inlineStr">
+        <is>
+          <t>SP02a, SP02b, SP02c, SP02d, SP02e, SP02f</t>
         </is>
       </c>
     </row>
@@ -7339,14 +7723,14 @@
           <t>Estruturas e Decisões Analisadas em createPlan()</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="21" t="n"/>
+      <c r="H3" s="21" t="n"/>
+      <c r="I3" s="22" t="n"/>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
@@ -9503,6 +9887,1915 @@
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>SPRINT 6 — Duplos de Teste: Stubs e Mocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>Contexto — Escolha dos Duplos</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="21" t="n"/>
+      <c r="H3" s="22" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Duplo</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Direcção</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Propósito</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Justificação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>TemperatureGatewayStub</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>temperatureGateway</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>Gateway → App (entrada)</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
+        <is>
+          <t>Fornecer dados controlados</t>
+        </is>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>Medição automática: app RECEBE dados do sensor. Stub substitui o sensor sem hardware real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="39" t="inlineStr">
+        <is>
+          <t>NotificationGatewayMock</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>notificationGateway</t>
+        </is>
+      </c>
+      <c r="D6" s="39" t="inlineStr">
+        <is>
+          <t>App → Gateway (saída)</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>Verificar que foi chamado</t>
+        </is>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>Envio de notificação: app ENVIA para o exterior. Mock verifica que a chamada foi feita com os args corretos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>Testes com Stub — TemperatureGateway (fornece dados pré-definidos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H10" s="41" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>SP01a</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. normal → sem alerta</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 23 (dentro dos limites)</t>
+        </is>
+      </c>
+      <c r="G11" s="38" t="inlineStr">
+        <is>
+          <t>alert=null, notified=false, sendNotification NÃO chamado</t>
+        </is>
+      </c>
+      <c r="H11" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>SP01b</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. acima → alerta Aviso</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 30 (acima de 28)</t>
+        </is>
+      </c>
+      <c r="G12" s="38" t="inlineStr">
+        <is>
+          <t>alert.classification='Aviso', notified=true</t>
+        </is>
+      </c>
+      <c r="H12" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>SP01c</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. crítica → alerta Critico</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 34 (acima de maxTemp+5)</t>
+        </is>
+      </c>
+      <c r="G13" s="38" t="inlineStr">
+        <is>
+          <t>alert.classification='Critico', notified=true</t>
+        </is>
+      </c>
+      <c r="H13" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
+          <t>SP01d</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. abaixo → alerta Aviso</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 10 (abaixo de 18)</t>
+        </is>
+      </c>
+      <c r="G14" s="38" t="inlineStr">
+        <is>
+          <t>alert not null, notified=true</t>
+        </is>
+      </c>
+      <c r="H14" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>SP01e</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: gateway falha → erro propagado</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → rejects('Sensor indisponível')</t>
+        </is>
+      </c>
+      <c r="G15" s="38" t="inlineStr">
+        <is>
+          <t>Lança erro 'Sensor indisponível'</t>
+        </is>
+      </c>
+      <c r="H15" s="38" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t>Testes com Mock — NotificationGateway (verifica chamadas e argumentos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E19" s="43" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F19" s="43" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G19" s="43" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H19" s="43" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>SP02a</t>
+        </is>
+      </c>
+      <c r="B20" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: alerta → notificação enviada ao admin</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D20" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E20" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>temp=30 (Stub), sendNotification.mockResolvedValue(true)</t>
+        </is>
+      </c>
+      <c r="G20" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado 1x com recipient='admin@greenherb.pt'</t>
+        </is>
+      </c>
+      <c r="H20" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>SP02b</t>
+        </is>
+      </c>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: sem alerta → notificação NÃO enviada</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>temp=23 (Stub), sendNotification.mockResolvedValue(true)</t>
+        </is>
+      </c>
+      <c r="G21" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification NÃO chamado (toHaveBeenCalledTimes(0))</t>
+        </is>
+      </c>
+      <c r="H21" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>SP02c</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: alerta Critico → subject contém 'Critico'</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E22" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>temp=34 (Stub), sendNotification.mockResolvedValue(true)</t>
+        </is>
+      </c>
+      <c r="G22" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado com subject contendo 'Critico'</t>
+        </is>
+      </c>
+      <c r="H22" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>SP02d</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: alerta Aviso → subject contém 'Aviso'</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>temp=30 (Stub), sendNotification.mockResolvedValue(true)</t>
+        </is>
+      </c>
+      <c r="G23" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado com subject contendo 'Aviso'</t>
+        </is>
+      </c>
+      <c r="H23" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>SP02e</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: falha notificação → erro propagado</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D24" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E24" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification.mockRejectedValue('Serviço indisponível')</t>
+        </is>
+      </c>
+      <c r="G24" s="39" t="inlineStr">
+        <is>
+          <t>Lança erro 'Serviço de notificações indisponível'</t>
+        </is>
+      </c>
+      <c r="H24" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>SP02f</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: múltiplas leituras → 2 notificações</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService interno)</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E25" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>temp=30,23,31 (Stub sequencial)</t>
+        </is>
+      </c>
+      <c r="G25" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado exatamente 2x</t>
+        </is>
+      </c>
+      <c r="H25" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna sequência</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>Diferença entre Stub e Mock</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Critério</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Stub (TemperatureGateway)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Mock (NotificationGateway)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Propósito</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>Fornecer dados controlados</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Verificar que foi chamado</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Direcção</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Gateway → App (entrada)</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>App → Gateway (saída)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>O que verifica</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Comportamento da app com esses dados</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>Se a chamada foi feita corretamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Exemplo</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature() devolve 30</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification() chamado com recipient correto</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>jest.fn().mockResolvedValue(30)</t>
+        </is>
+      </c>
+      <c r="C34" s="39" t="inlineStr">
+        <is>
+          <t>expect(fn).toHaveBeenCalledWith(...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="25" customHeight="1">
+      <c r="A37" s="35" t="inlineStr">
+        <is>
+          <t>Cobertura — Sprint 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Ficheiro</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Instruções</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Ramos</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Funções</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Linhas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>monitoringService.js</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>temperatureGateway.js</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>notificationGateway.js</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>71.34%</t>
+        </is>
+      </c>
+      <c r="C42" s="18" t="inlineStr">
+        <is>
+          <t>91.7%</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>52.23%</t>
+        </is>
+      </c>
+      <c r="E42" s="18" t="inlineStr">
+        <is>
+          <t>72.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>Total de Testes</t>
+        </is>
+      </c>
+      <c r="B44" s="20" t="inlineStr">
+        <is>
+          <t>219 / 219 passaram</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>SPRINT 6 — Duplos de Teste: Stubs e Mocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
+      <c r="A3" s="44" t="inlineStr">
+        <is>
+          <t>Duplos Criados</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="45" t="inlineStr">
+        <is>
+          <t>Duplo</t>
+        </is>
+      </c>
+      <c r="B4" s="45" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C4" s="45" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>Direcção</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="inlineStr">
+        <is>
+          <t>Justificação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>TemperatureGatewayStub</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>temperatureGateway</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>Gateway → App (entrada)</t>
+        </is>
+      </c>
+      <c r="E5" s="38" t="inlineStr">
+        <is>
+          <t>A medição de temperatura é automática — a app RECEBE dados do sensor. O Stub substitui o sensor devolvendo valores controlados sem precisar de hardware real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="39" t="inlineStr">
+        <is>
+          <t>NotificationGatewayMock</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>notificationGateway</t>
+        </is>
+      </c>
+      <c r="D6" s="39" t="inlineStr">
+        <is>
+          <t>App → Gateway (saída)</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>O envio de notificações é uma ação da app para o exterior. O Mock VERIFICA que a notificação foi enviada corretamente com os argumentos certos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>Testes com Stub — TemperatureGateway (SP01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H10" s="41" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>SP01a</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. normal → sem alerta</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 23</t>
+        </is>
+      </c>
+      <c r="G11" s="38" t="inlineStr">
+        <is>
+          <t>alert=null, notified=false, sendNotification NÃO chamado</t>
+        </is>
+      </c>
+      <c r="H11" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>SP01b</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. acima → alerta Aviso</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F12" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 30</t>
+        </is>
+      </c>
+      <c r="G12" s="38" t="inlineStr">
+        <is>
+          <t>alert.classification='Aviso', notified=true</t>
+        </is>
+      </c>
+      <c r="H12" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>SP01c</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. crítica → alerta Critico</t>
+        </is>
+      </c>
+      <c r="C13" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 34</t>
+        </is>
+      </c>
+      <c r="G13" s="38" t="inlineStr">
+        <is>
+          <t>alert.classification='Critico', notified=true</t>
+        </is>
+      </c>
+      <c r="H13" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
+          <t>SP01d</t>
+        </is>
+      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: temp. abaixo → alerta Aviso</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E14" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F14" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → 10</t>
+        </is>
+      </c>
+      <c r="G14" s="38" t="inlineStr">
+        <is>
+          <t>alert not null, notified=true</t>
+        </is>
+      </c>
+      <c r="H14" s="38" t="inlineStr">
+        <is>
+          <t>Plan com limites [18-28]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="38" t="inlineStr">
+        <is>
+          <t>SP01e</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>RN-25: gateway falha → erro propagado</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E15" s="38" t="inlineStr">
+        <is>
+          <t>Stub</t>
+        </is>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature → rejects('Sensor indisponível')</t>
+        </is>
+      </c>
+      <c r="G15" s="38" t="inlineStr">
+        <is>
+          <t>Lança erro 'Sensor indisponível'</t>
+        </is>
+      </c>
+      <c r="H15" s="38" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t>Testes com Mock — NotificationGateway (SP02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Requisito / Regra</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="D19" s="43" t="inlineStr">
+        <is>
+          <t>Nível</t>
+        </is>
+      </c>
+      <c r="E19" s="43" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="F19" s="43" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="G19" s="43" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="H19" s="43" t="inlineStr">
+        <is>
+          <t>Pré-condições</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>SP02a</t>
+        </is>
+      </c>
+      <c r="B20" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: alerta → notificação enviada ao admin</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D20" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E20" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F20" s="39" t="inlineStr">
+        <is>
+          <t>temp=30</t>
+        </is>
+      </c>
+      <c r="G20" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado 1x com recipient='admin@greenherb.pt'</t>
+        </is>
+      </c>
+      <c r="H20" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>SP02b</t>
+        </is>
+      </c>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: sem alerta → notificação NÃO enviada</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F21" s="39" t="inlineStr">
+        <is>
+          <t>temp=23</t>
+        </is>
+      </c>
+      <c r="G21" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification NÃO chamado</t>
+        </is>
+      </c>
+      <c r="H21" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>SP02c</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: alerta Critico → subject contém 'Critico'</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E22" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F22" s="39" t="inlineStr">
+        <is>
+          <t>temp=34</t>
+        </is>
+      </c>
+      <c r="G22" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado com subject contendo 'Critico'</t>
+        </is>
+      </c>
+      <c r="H22" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>SP02d</t>
+        </is>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: alerta Aviso → subject contém 'Aviso'</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>temp=30</t>
+        </is>
+      </c>
+      <c r="G23" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado com subject contendo 'Aviso'</t>
+        </is>
+      </c>
+      <c r="H23" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>SP02e</t>
+        </is>
+      </c>
+      <c r="B24" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: falha notificação → erro propagado</t>
+        </is>
+      </c>
+      <c r="C24" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D24" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E24" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F24" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification rejects</t>
+        </is>
+      </c>
+      <c r="G24" s="39" t="inlineStr">
+        <is>
+          <t>Lança erro 'Serviço de notificações indisponível'</t>
+        </is>
+      </c>
+      <c r="H24" s="39" t="inlineStr">
+        <is>
+          <t>Stub retorna 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>SP02f</t>
+        </is>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>RN-26: múltiplas leituras → 2 notificações</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>(monitoringService)</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>Unidade</t>
+        </is>
+      </c>
+      <c r="E25" s="39" t="inlineStr">
+        <is>
+          <t>Mock</t>
+        </is>
+      </c>
+      <c r="F25" s="39" t="inlineStr">
+        <is>
+          <t>temp=30,23,31 (sequência)</t>
+        </is>
+      </c>
+      <c r="G25" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification chamado exatamente 2x</t>
+        </is>
+      </c>
+      <c r="H25" s="39" t="inlineStr">
+        <is>
+          <t>Stub sequência</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25" customHeight="1">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>Diferença entre Stub e Mock</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="25" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Critério</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Stub (TemperatureGateway)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Mock (NotificationGateway)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Propósito</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>Fornecer dados controlados</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Verificar que foi chamado</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Direcção</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Gateway → App (entrada)</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>App → Gateway (saída)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>O que verifica</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Comportamento da app com os dados recebidos</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>Se a chamada foi feita corretamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Exemplo</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>getTemperature() devolve 30</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>sendNotification() foi chamado com recipient correto</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="25" customHeight="1">
+      <c r="A36" s="35" t="inlineStr">
+        <is>
+          <t>Cobertura — Sprint 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="25" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Ficheiro</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Instruções</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Ramos</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Funções</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Linhas</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>monitoringService.js</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>temperatureGateway.js</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>notificationGateway.js</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>66.66%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
+        <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t>71.34%</t>
+        </is>
+      </c>
+      <c r="C41" s="18" t="inlineStr">
+        <is>
+          <t>91.7%</t>
+        </is>
+      </c>
+      <c r="D41" s="18" t="inlineStr">
+        <is>
+          <t>52.23%</t>
+        </is>
+      </c>
+      <c r="E41" s="18" t="inlineStr">
+        <is>
+          <t>72.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Total de Testes</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>219 / 219 passaram</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>